<commit_message>
docs: endpointing timers parked at the cap, LiveKit left to govern
Second round. Raising the timers to 1/2/2 was not enough — the turn still
split after a thinking pause longer than two seconds, mid-sentence, which
is normal speech and not something any fixed silence timer can read.

So the aim changed: instead of tuning the dumb timers upward, park them at
their ceiling and get them out of the way, leaving LiveKit's smart
endpointing as the binding constraint. Its wait function floors at 2s and
rises to 6s when it judges the speaker is still going — a judgement made
on the words, which is the thing a silence timer cannot do.

Vapi caps all three at 3 seconds; 5 comes back as a 400. That cap is
itself a hint that the platform expects smart endpointing to cover
anything longer.

Now 3/3/3, provider livekit, waitFunction unchanged. Verified by re-read.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LvWpcUjn8Q7usdzv5KjT3N
</commit_message>
<xml_diff>
--- a/voice-assist/docs/Charlie-Voice-Settings-Tracker.xlsx
+++ b/voice-assist/docs/Charlie-Voice-Settings-Tracker.xlsx
@@ -1368,32 +1368,112 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="21" t="n"/>
-      <c r="B8" s="21" t="n"/>
-      <c r="C8" s="21" t="n"/>
-      <c r="D8" s="21" t="n"/>
-      <c r="E8" s="21" t="n"/>
+      <c r="A8" s="16" t="inlineStr">
+        <is>
+          <t>13/08/26</t>
+        </is>
+      </c>
+      <c r="B8" s="16" t="inlineStr">
+        <is>
+          <t>onPunctuationSeconds</t>
+        </is>
+      </c>
+      <c r="C8" s="16" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D8" s="16" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="E8" s="16" t="inlineStr">
+        <is>
+          <t>Raised to the CAP. Vapi rejects anything over 3s (400: "must not be greater than 3").</t>
+        </is>
+      </c>
     </row>
     <row r="9">
-      <c r="A9" s="21" t="n"/>
-      <c r="B9" s="21" t="n"/>
-      <c r="C9" s="21" t="n"/>
-      <c r="D9" s="21" t="n"/>
-      <c r="E9" s="21" t="n"/>
+      <c r="A9" s="16" t="inlineStr">
+        <is>
+          <t>13/08/26</t>
+        </is>
+      </c>
+      <c r="B9" s="16" t="inlineStr">
+        <is>
+          <t>onNoPunctuationSeconds</t>
+        </is>
+      </c>
+      <c r="C9" s="16" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D9" s="16" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="E9" s="16" t="inlineStr">
+        <is>
+          <t>same edit</t>
+        </is>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" s="21" t="n"/>
-      <c r="B10" s="21" t="n"/>
-      <c r="C10" s="21" t="n"/>
-      <c r="D10" s="21" t="n"/>
-      <c r="E10" s="21" t="n"/>
+      <c r="A10" s="16" t="inlineStr">
+        <is>
+          <t>13/08/26</t>
+        </is>
+      </c>
+      <c r="B10" s="16" t="inlineStr">
+        <is>
+          <t>onNumberSeconds</t>
+        </is>
+      </c>
+      <c r="C10" s="16" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D10" s="16" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="E10" s="16" t="inlineStr">
+        <is>
+          <t>same edit</t>
+        </is>
+      </c>
     </row>
     <row r="11">
-      <c r="A11" s="21" t="n"/>
-      <c r="B11" s="21" t="n"/>
-      <c r="C11" s="21" t="n"/>
-      <c r="D11" s="21" t="n"/>
-      <c r="E11" s="21" t="n"/>
+      <c r="A11" s="16" t="inlineStr">
+        <is>
+          <t>13/08/26</t>
+        </is>
+      </c>
+      <c r="B11" s="16" t="inlineStr">
+        <is>
+          <t>(rationale)</t>
+        </is>
+      </c>
+      <c r="C11" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D11" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E11" s="16" t="inlineStr">
+        <is>
+          <t>Deliberate: park the dumb timers at their ceiling so LiveKit smart endpointing becomes the governing constraint. Its curve floors at 2s and rises to 6s when it judges you are still speaking — which no fixed silence timer can do. Turn was still splitting after a &gt;2s thinking pause mid-sentence, so bigger fixed timers were the wrong tool.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="21" t="n"/>

</xml_diff>

<commit_message>
docs: log the backoff fix and where tonight landed
backoffSeconds 0.8 -> 3. Charlie was being interrupted correctly at two
words and then barging straight back in eight-tenths of a second later,
while Steven was still mid-sentence, getting cut off again, and cycling.
That was the listening/speaking ping-pong he could see on screen — real
speech, not the label bug fixed alongside it.

Also records what is still open: the "Meeting has ended" drops seen on a
phone in the red battery zone (not chased — suspect iOS power management,
worth re-testing on a charged phone), empty Deepgram keywords, and the
ambient background WAV.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LvWpcUjn8Q7usdzv5KjT3N
</commit_message>
<xml_diff>
--- a/voice-assist/docs/Charlie-Voice-Settings-Tracker.xlsx
+++ b/voice-assist/docs/Charlie-Voice-Settings-Tracker.xlsx
@@ -1476,25 +1476,85 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="21" t="n"/>
-      <c r="B12" s="21" t="n"/>
-      <c r="C12" s="21" t="n"/>
-      <c r="D12" s="21" t="n"/>
-      <c r="E12" s="21" t="n"/>
+      <c r="A12" s="16" t="inlineStr">
+        <is>
+          <t>13/08/26</t>
+        </is>
+      </c>
+      <c r="B12" s="16" t="inlineStr">
+        <is>
+          <t>stopSpeakingPlan.backoffSeconds</t>
+        </is>
+      </c>
+      <c r="C12" s="16" t="inlineStr">
+        <is>
+          <t>0.8</t>
+        </is>
+      </c>
+      <c r="D12" s="16" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="E12" s="16" t="inlineStr">
+        <is>
+          <t>The ping-pong. Charlie was interrupted correctly at 2 words, then barged back in 0.8s later while Steven was still mid-sentence, got cut off again, and cycled. Now stays down 3s once interrupted.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
-      <c r="A13" s="21" t="n"/>
-      <c r="B13" s="21" t="n"/>
-      <c r="C13" s="21" t="n"/>
-      <c r="D13" s="21" t="n"/>
-      <c r="E13" s="21" t="n"/>
+      <c r="A13" s="16" t="inlineStr">
+        <is>
+          <t>13/08/26</t>
+        </is>
+      </c>
+      <c r="B13" s="16" t="inlineStr">
+        <is>
+          <t>(app) speaking-label debounce</t>
+        </is>
+      </c>
+      <c r="C13" s="16" t="inlineStr">
+        <is>
+          <t>instant</t>
+        </is>
+      </c>
+      <c r="D13" s="16" t="inlineStr">
+        <is>
+          <t>350ms</t>
+        </is>
+      </c>
+      <c r="E13" s="16" t="inlineStr">
+        <is>
+          <t>UI only. Empty speech turns for held-back fragments were rendering as SPEAKING. Label was lying; mic never stopped.</t>
+        </is>
+      </c>
     </row>
     <row r="14">
-      <c r="A14" s="21" t="n"/>
-      <c r="B14" s="21" t="n"/>
-      <c r="C14" s="21" t="n"/>
-      <c r="D14" s="21" t="n"/>
-      <c r="E14" s="21" t="n"/>
+      <c r="A14" s="16" t="inlineStr">
+        <is>
+          <t>13/08/26</t>
+        </is>
+      </c>
+      <c r="B14" s="16" t="inlineStr">
+        <is>
+          <t>(observed)</t>
+        </is>
+      </c>
+      <c r="C14" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D14" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E14" s="16" t="inlineStr">
+        <is>
+          <t>Fragments still split into bubbles but Charlie now answers the whole thought once — the goal. Remaining: "Voice error - Meeting has ended" seen twice on a phone in the red battery zone; not chased, suspect iOS power management. Deepgram keywords still empty (Marites -&gt; "many tiers"). backgroundSound ambient WAV still on.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>